<commit_message>
object classes, django 6.1
</commit_message>
<xml_diff>
--- a/app_kit/tests/TESTS_ROOT/xlsx_for_testing/TaxonProfiles/valid_partial_update/Taxon profiles.xlsx
+++ b/app_kit/tests/TESTS_ROOT/xlsx_for_testing/TaxonProfiles/valid_partial_update/Taxon profiles.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Taxon Profiles" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
   <si>
     <t xml:space="preserve">Scientific Name</t>
   </si>
@@ -88,30 +88,6 @@
   </si>
   <si>
     <t xml:space="preserve">Primary image (optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leaf.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art Vandeley</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC BY-SA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://imageworld.com/lacerta-agilis.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leaf title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leaf caption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leaf alt text</t>
   </si>
   <si>
     <t xml:space="preserve">URL</t>
@@ -441,37 +417,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -3766,30 +3742,14 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>29</v>
-      </c>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
       <c r="I2" s="8"/>
     </row>
   </sheetData>
@@ -3819,19 +3779,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>19</v>
@@ -3848,31 +3808,31 @@
         <v>6</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E2" s="8"/>
       <c r="F2" s="8" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
@@ -3880,13 +3840,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
@@ -3895,13 +3855,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
@@ -3910,13 +3870,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
@@ -3925,13 +3885,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>

</xml_diff>